<commit_message>
Major repository update - rename scripts, update figures and tables
Scripts:
- Renamed all figure scripts from v2/v3 to v1 for consistency
- Removed FigS1 (network resistance class) - not included in manuscript
- Added figS5_regression_residuals_v1.R

Figures:
- Removed FigS1 (eliminated from manuscript)
- Renamed FigS2-S5 to FigS1-S4 to match new numbering
- Updated Fig2: replaced □ symbol with * for robust trend genes
- Updated Fig3: corrected n values (Human=6,549, Animal=236, Env=377)
- Updated Fig4: corrected n values
- Updated FigS2 (now FigS2): fixed NaN row, alignment, legend position

Tables:
- TableS6/S7: removed NaN country row (37/95 countries)
- TableS12: added XLSX version
- Updated TableS12 with correct NMI Louvain-Infomap = 0.784
</commit_message>
<xml_diff>
--- a/results/supplementary/tables_submission/TableS7_whitelist_genes_by_country.xlsx
+++ b/results/supplementary/tables_submission/TableS7_whitelist_genes_by_country.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TableS7_whitelist_genes_by_coun" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -73,9 +73,7 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -443,25 +441,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P97"/>
+  <dimension ref="A1:P96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1941,25 +1939,29 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>49</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1969,47 +1971,47 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
           <t>2</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L19" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M19" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
         </is>
       </c>
       <c r="P19" s="3" t="inlineStr">
@@ -2021,69 +2023,69 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2091,39 +2093,39 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>121</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2133,7 +2135,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -2163,7 +2165,7 @@
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
@@ -2173,121 +2175,121 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>105</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>47</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>104</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>89</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2297,7 +2299,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -2337,121 +2339,121 @@
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>98</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>70</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>94</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2501,56 +2503,56 @@
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>91</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>67</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2588,36 +2590,36 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>86</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -2630,34 +2632,34 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -2670,34 +2672,34 @@
       </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>73</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Afghanistan</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>67</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2737,7 +2739,7 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -2752,34 +2754,34 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>72</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Afghanistan</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -2834,34 +2836,34 @@
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>70</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>55</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2911,39 +2913,39 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>66</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -2958,7 +2960,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2988,7 +2990,7 @@
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>13</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
@@ -3005,22 +3007,22 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>38</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3035,12 +3037,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3070,39 +3072,39 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>50</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -3117,7 +3119,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -3157,29 +3159,29 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3189,7 +3191,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3229,7 +3231,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3244,24 +3246,24 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>42</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Sudan</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>29</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -3271,7 +3273,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -3311,49 +3313,49 @@
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N35" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>41</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Sudan</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3403,39 +3405,39 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>40</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Myanmar</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -3485,29 +3487,29 @@
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P37" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>38</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Myanmar</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3517,7 +3519,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3572,24 +3574,24 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>36</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3599,7 +3601,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -3654,24 +3656,24 @@
       </c>
       <c r="P39" s="3" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3681,7 +3683,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3736,34 +3738,34 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Kosovo</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3818,14 +3820,14 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Kosovo</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -3835,12 +3837,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -3907,22 +3909,22 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -3982,34 +3984,34 @@
       </c>
       <c r="P43" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4059,7 +4061,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -4071,24 +4073,24 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
           <t>2</t>
@@ -4141,7 +4143,7 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
@@ -4153,7 +4155,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4163,7 +4165,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -4173,7 +4175,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -4223,7 +4225,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -4235,7 +4237,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -4245,12 +4247,12 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -4310,29 +4312,29 @@
       </c>
       <c r="P47" s="3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -4392,106 +4394,106 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Libya</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O49" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="P49" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Libya</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -4501,7 +4503,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -4541,7 +4543,7 @@
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4551,39 +4553,39 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -4623,7 +4625,7 @@
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N51" s="3" t="inlineStr">
@@ -4638,84 +4640,84 @@
       </c>
       <c r="P51" s="3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O52" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -4727,22 +4729,22 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -4797,7 +4799,7 @@
       </c>
       <c r="O53" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P53" s="3" t="inlineStr">
@@ -4809,104 +4811,104 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
         <is>
           <t>14</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O54" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P54" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Togo</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -4973,29 +4975,29 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Togo</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -5048,34 +5050,34 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Montenegro</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -5137,27 +5139,27 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Montenegro</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -5197,7 +5199,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -5212,66 +5214,66 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -5279,7 +5281,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -5301,27 +5303,27 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -5351,7 +5353,7 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -5383,54 +5385,54 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -5458,36 +5460,36 @@
       </c>
       <c r="P61" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -5510,7 +5512,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5547,17 +5549,17 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -5567,7 +5569,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -5622,14 +5624,14 @@
       </c>
       <c r="P63" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -5639,17 +5641,17 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -5704,14 +5706,14 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -5721,17 +5723,17 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -5793,17 +5795,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Tanzania</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5868,24 +5870,24 @@
       </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Tanzania</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -5957,17 +5959,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -6039,19 +6041,19 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -6059,7 +6061,7 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -6114,24 +6116,24 @@
       </c>
       <c r="P69" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Cote d'Ivoire</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -6141,7 +6143,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -6203,27 +6205,27 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Cote d'Ivoire</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -6258,7 +6260,7 @@
       </c>
       <c r="L71" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M71" s="3" t="inlineStr">
@@ -6278,14 +6280,14 @@
       </c>
       <c r="P71" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -6300,7 +6302,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -6340,7 +6342,7 @@
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
@@ -6367,7 +6369,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -6377,17 +6379,17 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -6449,7 +6451,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -6469,7 +6471,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -6524,14 +6526,14 @@
       </c>
       <c r="P74" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -6541,37 +6543,37 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
           <t>4</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F75" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G75" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H75" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I75" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
@@ -6613,7 +6615,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -6623,12 +6625,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -6653,7 +6655,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -6695,104 +6697,104 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P77" s="3" t="inlineStr">
+        <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O77" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P77" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Honduras</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -6859,12 +6861,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Benin</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -6874,12 +6876,12 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -6941,19 +6943,19 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Benin</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -6961,57 +6963,57 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O80" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="P80" s="2" t="inlineStr">
@@ -7023,7 +7025,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Belarus</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -7033,14 +7035,14 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -7093,7 +7095,7 @@
       </c>
       <c r="O81" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P81" s="3" t="inlineStr">
@@ -7105,7 +7107,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -7115,79 +7117,79 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
           <t>2</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O82" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P82" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -7197,12 +7199,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
           <t>2</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
@@ -7269,7 +7271,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -7279,12 +7281,12 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -7351,7 +7353,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -7361,12 +7363,12 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
@@ -7433,12 +7435,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Djibouti</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -7448,7 +7450,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -7515,89 +7517,89 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Djibouti</t>
+          <t>Sydney</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C87" s="3" t="inlineStr">
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O87" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P87" s="3" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O87" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P87" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Not collected</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -7679,7 +7681,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Not collected</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -7689,12 +7691,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -7761,7 +7763,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Albania</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -7771,12 +7773,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -7843,7 +7845,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Albania</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -7925,17 +7927,17 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Ethiopia</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -8007,7 +8009,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
+          <t>Rwanda</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -8089,17 +8091,17 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -8171,7 +8173,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -8253,7 +8255,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>North Korea</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -8327,88 +8329,6 @@
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>North Korea</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O97" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P97" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>